<commit_message>
first draft - after first revidsion
Main revision
</commit_message>
<xml_diff>
--- a/Cielo2025/NewMask_052025/LiNbO3 - Cielo - TO#2 - 001.xlsx
+++ b/Cielo2025/NewMask_052025/LiNbO3 - Cielo - TO#2 - 001.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iengel\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\db\Documents\GitHub\BorisLab\Cielo2025\NewMask_052025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A91678-A0AD-4B6C-9182-D5DFF2B179E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1640224-9E7C-4E48-96EE-9111B074F558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{63A053E8-0D7E-4E7E-9D73-CB3A018A5259}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{63A053E8-0D7E-4E7E-9D73-CB3A018A5259}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="36">
   <si>
     <t>SN</t>
   </si>
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -332,15 +332,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -350,37 +341,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -389,11 +365,32 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -784,49 +781,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729037F2-56C6-4358-9EA4-6699D0628A9B}">
   <dimension ref="A1:I58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" style="9" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="6" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.28515625" customWidth="1"/>
-    <col min="8" max="8" width="12" style="9" customWidth="1"/>
-    <col min="9" max="9" width="41.85546875" customWidth="1"/>
+    <col min="5" max="5" width="24.26953125" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.26953125" customWidth="1"/>
+    <col min="8" max="8" width="12" style="6" customWidth="1"/>
+    <col min="9" max="9" width="41.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="25" t="s">
+      <c r="F1" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="I1" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="19">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="11">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -847,13 +844,13 @@
       <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="19">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="11">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -874,13 +871,13 @@
       <c r="G3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="22">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -906,8 +903,8 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="23"/>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
@@ -926,11 +923,11 @@
       <c r="G5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="24"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="22">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -956,8 +953,8 @@
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="21"/>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="23"/>
       <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
@@ -976,14 +973,14 @@
       <c r="G7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="18"/>
+      <c r="H7" s="24"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="19">
-        <v>5</v>
-      </c>
-      <c r="B8" s="5" t="s">
+    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="11">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -1001,18 +998,18 @@
       <c r="G8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="19">
+    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -1030,18 +1027,18 @@
       <c r="G9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="I9" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="19">
+    <row r="10" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="11">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -1059,18 +1056,18 @@
       <c r="G10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="19">
+    <row r="11" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="11">
         <v>8</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1088,18 +1085,18 @@
       <c r="G11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="19">
-        <v>9</v>
-      </c>
-      <c r="B12" s="5" t="s">
+    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="11">
+        <v>9</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -1117,18 +1114,18 @@
       <c r="G12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H12" s="14" t="s">
+      <c r="H12" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="19">
+    <row r="13" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="11">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -1146,18 +1143,18 @@
       <c r="G13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="14" t="s">
+      <c r="H13" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="19">
-        <v>11</v>
-      </c>
-      <c r="B14" s="5" t="s">
+    <row r="14" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="11">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -1175,18 +1172,18 @@
       <c r="G14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="19">
-        <v>12</v>
-      </c>
-      <c r="B15" s="5" t="s">
+    <row r="15" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="11">
+        <v>12</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -1204,15 +1201,15 @@
       <c r="G15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="19">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="11">
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1233,13 +1230,13 @@
       <c r="G16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="13" t="s">
+      <c r="H16" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="19">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="11">
         <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1260,13 +1257,13 @@
       <c r="G17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="13" t="s">
+      <c r="H17" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="19">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="11">
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1287,13 +1284,13 @@
       <c r="G18" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="19">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="11">
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -1314,13 +1311,13 @@
       <c r="G19" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="13" t="s">
+      <c r="H19" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I19" s="4"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="11">
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1341,13 +1338,13 @@
       <c r="G20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I20" s="4"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="19">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="11">
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -1368,43 +1365,67 @@
       <c r="G21" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="H21" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="19">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="11">
         <v>19</v>
       </c>
-      <c r="B22" s="3"/>
+      <c r="B22" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="C22" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
+      <c r="D22" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>27</v>
+      </c>
       <c r="I22" s="4"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="19">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="11">
         <v>20</v>
       </c>
-      <c r="B23" s="3"/>
+      <c r="B23" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="C23" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
+      <c r="D23" s="2">
+        <v>5</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>27</v>
+      </c>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="22">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="14">
         <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1428,12 +1449,12 @@
       <c r="H24" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="11" t="s">
+      <c r="I24" s="21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="23"/>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="15"/>
       <c r="B25" s="1" t="s">
         <v>7</v>
       </c>
@@ -1452,11 +1473,11 @@
       <c r="G25" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="22">
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="14">
         <v>22</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -1480,12 +1501,12 @@
       <c r="H26" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I26" s="11" t="s">
+      <c r="I26" s="21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="23"/>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="15"/>
       <c r="B27" s="1" t="s">
         <v>7</v>
       </c>
@@ -1504,11 +1525,11 @@
       <c r="G27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="22">
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="14">
         <v>23</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -1532,12 +1553,12 @@
       <c r="H28" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I28" s="11" t="s">
+      <c r="I28" s="21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="23"/>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" s="15"/>
       <c r="B29" s="1" t="s">
         <v>7</v>
       </c>
@@ -1556,11 +1577,11 @@
       <c r="G29" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H29" s="12"/>
-      <c r="I29" s="12"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="22">
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" s="14">
         <v>24</v>
       </c>
       <c r="B30" s="3" t="s">
@@ -1584,12 +1605,12 @@
       <c r="H30" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I30" s="6" t="s">
+      <c r="I30" s="19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="23"/>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="15"/>
       <c r="B31" s="3" t="s">
         <v>19</v>
       </c>
@@ -1608,11 +1629,11 @@
       <c r="G31" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H31" s="12"/>
-      <c r="I31" s="7"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="22">
+      <c r="H31" s="17"/>
+      <c r="I31" s="20"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="14">
         <v>25</v>
       </c>
       <c r="B32" s="3" t="s">
@@ -1636,12 +1657,12 @@
       <c r="H32" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I32" s="19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="23"/>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="15"/>
       <c r="B33" s="3" t="s">
         <v>19</v>
       </c>
@@ -1660,11 +1681,11 @@
       <c r="G33" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H33" s="12"/>
-      <c r="I33" s="7"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="22">
+      <c r="H33" s="17"/>
+      <c r="I33" s="20"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="14">
         <v>26</v>
       </c>
       <c r="B34" s="3" t="s">
@@ -1688,12 +1709,12 @@
       <c r="H34" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I34" s="6" t="s">
+      <c r="I34" s="19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="23"/>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="15"/>
       <c r="B35" s="3" t="s">
         <v>19</v>
       </c>
@@ -1712,11 +1733,11 @@
       <c r="G35" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H35" s="12"/>
-      <c r="I35" s="7"/>
-    </row>
-    <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A36" s="24">
+      <c r="H35" s="17"/>
+      <c r="I35" s="20"/>
+    </row>
+    <row r="36" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" s="12">
         <v>27</v>
       </c>
       <c r="B36" s="3" t="s">
@@ -1737,15 +1758,15 @@
       <c r="G36" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H36" s="17" t="s">
+      <c r="H36" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I36" s="10" t="s">
+      <c r="I36" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="24">
+    <row r="37" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="12">
         <v>28</v>
       </c>
       <c r="B37" s="3" t="s">
@@ -1766,15 +1787,15 @@
       <c r="G37" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H37" s="17" t="s">
+      <c r="H37" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I37" s="10" t="s">
+      <c r="I37" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="24">
+    <row r="38" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A38" s="12">
         <v>29</v>
       </c>
       <c r="B38" s="3" t="s">
@@ -1795,15 +1816,15 @@
       <c r="G38" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H38" s="17" t="s">
+      <c r="H38" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I38" s="10" t="s">
+      <c r="I38" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="22">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="14">
         <v>30</v>
       </c>
       <c r="B39" s="3" t="s">
@@ -1824,15 +1845,15 @@
       <c r="G39" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H39" s="15" t="s">
+      <c r="H39" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I39" s="6" t="s">
+      <c r="I39" s="19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="23"/>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="15"/>
       <c r="B40" s="3" t="s">
         <v>24</v>
       </c>
@@ -1851,11 +1872,11 @@
       <c r="G40" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H40" s="12"/>
-      <c r="I40" s="7"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="22">
+      <c r="H40" s="17"/>
+      <c r="I40" s="20"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="14">
         <v>31</v>
       </c>
       <c r="B41" s="3" t="s">
@@ -1876,15 +1897,15 @@
       <c r="G41" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H41" s="15" t="s">
+      <c r="H41" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="I41" s="19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="23"/>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" s="15"/>
       <c r="B42" s="3" t="s">
         <v>24</v>
       </c>
@@ -1903,11 +1924,11 @@
       <c r="G42" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H42" s="12"/>
-      <c r="I42" s="7"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="22">
+      <c r="H42" s="17"/>
+      <c r="I42" s="20"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" s="14">
         <v>32</v>
       </c>
       <c r="B43" s="3" t="s">
@@ -1928,15 +1949,15 @@
       <c r="G43" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H43" s="15" t="s">
+      <c r="H43" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="I43" s="19" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="23"/>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" s="15"/>
       <c r="B44" s="3" t="s">
         <v>24</v>
       </c>
@@ -1955,11 +1976,11 @@
       <c r="G44" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H44" s="12"/>
-      <c r="I44" s="7"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="22">
+      <c r="H44" s="17"/>
+      <c r="I44" s="20"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" s="14">
         <v>33</v>
       </c>
       <c r="B45" s="3" t="s">
@@ -1980,13 +2001,13 @@
       <c r="G45" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H45" s="15" t="s">
+      <c r="H45" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I45" s="6"/>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="23"/>
+      <c r="I45" s="19"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46" s="15"/>
       <c r="B46" s="3" t="s">
         <v>24</v>
       </c>
@@ -2005,11 +2026,11 @@
       <c r="G46" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H46" s="12"/>
-      <c r="I46" s="7"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="22">
+      <c r="H46" s="17"/>
+      <c r="I46" s="20"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47" s="14">
         <v>34</v>
       </c>
       <c r="B47" s="3" t="s">
@@ -2030,13 +2051,13 @@
       <c r="G47" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H47" s="15" t="s">
+      <c r="H47" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I47" s="6"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="23"/>
+      <c r="I47" s="19"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48" s="15"/>
       <c r="B48" s="3" t="s">
         <v>24</v>
       </c>
@@ -2055,11 +2076,11 @@
       <c r="G48" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H48" s="12"/>
-      <c r="I48" s="7"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="22">
+      <c r="H48" s="17"/>
+      <c r="I48" s="20"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A49" s="14">
         <v>35</v>
       </c>
       <c r="B49" s="3" t="s">
@@ -2080,15 +2101,15 @@
       <c r="G49" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H49" s="15" t="s">
+      <c r="H49" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I49" s="6" t="s">
+      <c r="I49" s="19" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="23"/>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50" s="15"/>
       <c r="B50" s="3" t="s">
         <v>24</v>
       </c>
@@ -2107,11 +2128,11 @@
       <c r="G50" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H50" s="12"/>
-      <c r="I50" s="7"/>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="22">
+      <c r="H50" s="17"/>
+      <c r="I50" s="20"/>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51" s="14">
         <v>36</v>
       </c>
       <c r="B51" s="3" t="s">
@@ -2135,10 +2156,10 @@
       <c r="H51" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I51" s="6"/>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="23"/>
+      <c r="I51" s="19"/>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" s="15"/>
       <c r="B52" s="3" t="s">
         <v>24</v>
       </c>
@@ -2157,11 +2178,11 @@
       <c r="G52" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H52" s="12"/>
-      <c r="I52" s="7"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="22">
+      <c r="H52" s="17"/>
+      <c r="I52" s="20"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A53" s="14">
         <v>37</v>
       </c>
       <c r="B53" s="3" t="s">
@@ -2185,10 +2206,10 @@
       <c r="H53" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I53" s="6"/>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="23"/>
+      <c r="I53" s="19"/>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" s="15"/>
       <c r="B54" s="3" t="s">
         <v>24</v>
       </c>
@@ -2207,11 +2228,11 @@
       <c r="G54" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H54" s="12"/>
-      <c r="I54" s="7"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="22">
+      <c r="H54" s="17"/>
+      <c r="I54" s="20"/>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55" s="14">
         <v>38</v>
       </c>
       <c r="B55" s="3" t="s">
@@ -2237,8 +2258,8 @@
       </c>
       <c r="I55" s="4"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="23"/>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="15"/>
       <c r="B56" s="3" t="s">
         <v>24</v>
       </c>
@@ -2257,46 +2278,98 @@
       <c r="G56" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H56" s="12"/>
+      <c r="H56" s="17"/>
       <c r="I56" s="4"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="24">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A57" s="12">
         <v>39</v>
       </c>
-      <c r="B57" s="3"/>
+      <c r="B57" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C57" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D57" s="2">
         <v>5.5</v>
       </c>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="3"/>
+      <c r="E57" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H57" s="8" t="s">
+        <v>27</v>
+      </c>
       <c r="I57" s="4"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="24">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A58" s="12">
         <v>40</v>
       </c>
-      <c r="B58" s="3"/>
+      <c r="B58" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C58" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D58" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="3"/>
+        <v>5</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H58" s="8" t="s">
+        <v>27</v>
+      </c>
       <c r="I58" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I58" xr:uid="{729037F2-56C6-4358-9EA4-6699D0628A9B}"/>
   <mergeCells count="48">
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="H32:H33"/>
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="H41:H42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="I45:I46"/>
     <mergeCell ref="A55:A56"/>
     <mergeCell ref="H55:H56"/>
     <mergeCell ref="A43:A44"/>
@@ -2311,40 +2384,8 @@
     <mergeCell ref="I53:I54"/>
     <mergeCell ref="A51:A52"/>
     <mergeCell ref="A53:A54"/>
-    <mergeCell ref="H41:H42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="H45:H46"/>
     <mergeCell ref="H47:H48"/>
-    <mergeCell ref="I45:I46"/>
     <mergeCell ref="I47:I48"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="H32:H33"/>
-    <mergeCell ref="I32:I33"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="H34:H35"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="I30:I31"/>
-    <mergeCell ref="H30:H31"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="H28:H29"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H7"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>